<commit_message>
Refresh migration workbook from DemoCentral and DFactory
</commit_message>
<xml_diff>
--- a/cicd/migration_objects.xlsx
+++ b/cicd/migration_objects.xlsx
@@ -4600,7 +4600,7 @@
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>Ishita_SQL_Conn_Src</t>
+          <t>AA_ImportPolicyDAC_RestV2</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
@@ -4630,7 +4630,7 @@
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t>AA_ImportPolicyDAC_RestV2</t>
+          <t>cdp_rest_admin_export_user_groups</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
@@ -4652,7 +4652,7 @@
       <c r="F124" s="11" t="n"/>
       <c r="G124" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H124" s="11" t="n"/>
@@ -4660,7 +4660,7 @@
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t>cdp_dbx_rbac_permissions_uc_test</t>
+          <t>cdp_rest_cdam_create_access_control_policy</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
@@ -4682,7 +4682,7 @@
       <c r="F125" s="11" t="n"/>
       <c r="G125" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H125" s="11" t="n"/>
@@ -4690,7 +4690,7 @@
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t>cdp_flatfile_swaggerfile_debugging</t>
+          <t>cdp_rest_cdam_create_data_deidentification_policy</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
@@ -4712,7 +4712,7 @@
       <c r="F126" s="11" t="n"/>
       <c r="G126" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H126" s="11" t="n"/>
@@ -4720,7 +4720,7 @@
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
-          <t>cdp_flatfile_swaggerfile_templates</t>
+          <t>cdp_rest_cdam_create_data_filter_policy</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -4742,7 +4742,7 @@
       <c r="F127" s="11" t="n"/>
       <c r="G127" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H127" s="11" t="n"/>
@@ -4750,7 +4750,7 @@
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_admin_export_user_groups</t>
+          <t>cdp_rest_cdam_get_access_control_policies</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -4772,7 +4772,7 @@
       <c r="F128" s="11" t="n"/>
       <c r="G128" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H128" s="11" t="n"/>
@@ -4780,7 +4780,7 @@
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdam_create_access_control_policy</t>
+          <t>cdp_rest_cdam_get_data_deidentification_policies</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
@@ -4802,7 +4802,7 @@
       <c r="F129" s="11" t="n"/>
       <c r="G129" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H129" s="11" t="n"/>
@@ -4810,7 +4810,7 @@
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdam_create_data_deidentification_policy</t>
+          <t>cdp_rest_cdam_get_data_filter_policies</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
@@ -4832,7 +4832,7 @@
       <c r="F130" s="11" t="n"/>
       <c r="G130" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H130" s="11" t="n"/>
@@ -4840,7 +4840,7 @@
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdam_create_data_filter_policy</t>
+          <t>cdp_rest_cdgc_get_asset_details</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
@@ -4862,7 +4862,7 @@
       <c r="F131" s="11" t="n"/>
       <c r="G131" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H131" s="11" t="n"/>
@@ -4870,7 +4870,7 @@
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdam_get_access_control_policies</t>
+          <t>cdp_rest_cdgc_get_data_classification</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
@@ -4892,7 +4892,7 @@
       <c r="F132" s="11" t="n"/>
       <c r="G132" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H132" s="11" t="n"/>
@@ -4900,7 +4900,7 @@
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdam_get_data_deidentification_policies</t>
+          <t>cdp_rest_cdmp_add_data_assets_to_collection</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
@@ -4922,7 +4922,7 @@
       <c r="F133" s="11" t="n"/>
       <c r="G133" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H133" s="11" t="n"/>
@@ -4930,7 +4930,7 @@
     <row r="134">
       <c r="A134" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdam_get_data_filter_policies</t>
+          <t>cdp_rest_cdmp_get_assets_in_collections</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
@@ -4952,7 +4952,7 @@
       <c r="F134" s="11" t="n"/>
       <c r="G134" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H134" s="11" t="n"/>
@@ -4960,7 +4960,7 @@
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdgc_get_asset_details</t>
+          <t>cdp_rest_cdmp_get_data_collections</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
@@ -4982,7 +4982,7 @@
       <c r="F135" s="11" t="n"/>
       <c r="G135" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H135" s="11" t="n"/>
@@ -4990,7 +4990,7 @@
     <row r="136">
       <c r="A136" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdgc_get_data_classification</t>
+          <t>cdp_rest_idmc_generate_jwt_token</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
@@ -5012,7 +5012,7 @@
       <c r="F136" s="11" t="n"/>
       <c r="G136" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H136" s="11" t="n"/>
@@ -5020,7 +5020,7 @@
     <row r="137">
       <c r="A137" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdmp_add_data_assets_to_collection</t>
+          <t>cdp_rest_idmc_login_V2</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
@@ -5042,7 +5042,7 @@
       <c r="F137" s="11" t="n"/>
       <c r="G137" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H137" s="11" t="n"/>
@@ -5050,7 +5050,7 @@
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdmp_get_assets_in_collections</t>
+          <t>Cloud Integration Hub</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
@@ -5072,7 +5072,7 @@
       <c r="F138" s="11" t="n"/>
       <c r="G138" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H138" s="11" t="n"/>
@@ -5080,7 +5080,7 @@
     <row r="139">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_cdmp_get_data_collections</t>
+          <t>CON-AM-Project</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
@@ -5102,7 +5102,7 @@
       <c r="F139" s="11" t="n"/>
       <c r="G139" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H139" s="11" t="n"/>
@@ -5110,7 +5110,7 @@
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_idmc_generate_jwt_token</t>
+          <t>Ishita_SQL_Conn_Src</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
@@ -5132,7 +5132,7 @@
       <c r="F140" s="11" t="n"/>
       <c r="G140" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H140" s="11" t="n"/>
@@ -5140,7 +5140,7 @@
     <row r="141">
       <c r="A141" s="8" t="inlineStr">
         <is>
-          <t>cdp_rest_idmc_login_V2</t>
+          <t>RestV2-AM-Login</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
@@ -5162,7 +5162,7 @@
       <c r="F141" s="11" t="n"/>
       <c r="G141" s="12" t="inlineStr">
         <is>
-          <t>exists, in sync</t>
+          <t>exists, differs</t>
         </is>
       </c>
       <c r="H141" s="11" t="n"/>
@@ -5170,7 +5170,7 @@
     <row r="142">
       <c r="A142" s="8" t="inlineStr">
         <is>
-          <t>Cloud Integration Hub</t>
+          <t>cdp_dbx_rbac_permissions_uc_test</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
@@ -5200,7 +5200,7 @@
     <row r="143">
       <c r="A143" s="8" t="inlineStr">
         <is>
-          <t>CON-AM-Project</t>
+          <t>cdp_flatfile_swaggerfile_debugging</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
@@ -5230,7 +5230,7 @@
     <row r="144">
       <c r="A144" s="8" t="inlineStr">
         <is>
-          <t>conn-BM-Business</t>
+          <t>cdp_flatfile_swaggerfile_templates</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
@@ -5260,7 +5260,7 @@
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
-          <t>Conn-BM-FlatFile</t>
+          <t>conn-BM-Business</t>
         </is>
       </c>
       <c r="B145" s="10" t="inlineStr">
@@ -5290,7 +5290,7 @@
     <row r="146">
       <c r="A146" s="8" t="inlineStr">
         <is>
-          <t>Conn-BM-Flatfile-Pharma</t>
+          <t>Conn-BM-FlatFile</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
@@ -5320,7 +5320,7 @@
     <row r="147">
       <c r="A147" s="8" t="inlineStr">
         <is>
-          <t>conn_B2B_Inbound</t>
+          <t>Conn-BM-Flatfile-Pharma</t>
         </is>
       </c>
       <c r="B147" s="10" t="inlineStr">
@@ -5350,7 +5350,7 @@
     <row r="148">
       <c r="A148" s="8" t="inlineStr">
         <is>
-          <t>conn_BFSI_ Flatfile</t>
+          <t>conn_B2B_Inbound</t>
         </is>
       </c>
       <c r="B148" s="10" t="inlineStr">
@@ -5380,7 +5380,7 @@
     <row r="149">
       <c r="A149" s="8" t="inlineStr">
         <is>
-          <t>conn_ff_edf_8gg</t>
+          <t>conn_BFSI_ Flatfile</t>
         </is>
       </c>
       <c r="B149" s="10" t="inlineStr">
@@ -5410,7 +5410,7 @@
     <row r="150">
       <c r="A150" s="8" t="inlineStr">
         <is>
-          <t>dgov_dbx_rbac_permissions_pschp_dev_uc</t>
+          <t>conn_ff_edf_8gg</t>
         </is>
       </c>
       <c r="B150" s="10" t="inlineStr">
@@ -5440,7 +5440,7 @@
     <row r="151">
       <c r="A151" s="8" t="inlineStr">
         <is>
-          <t>DQ_Email_WSConsumer_EU_v1.4</t>
+          <t>dgov_dbx_rbac_permissions_pschp_dev_uc</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
@@ -5470,7 +5470,7 @@
     <row r="152">
       <c r="A152" s="8" t="inlineStr">
         <is>
-          <t>DQ_Email_WSConsumer_US_v1.4</t>
+          <t>DQ_Email_WSConsumer_EU_v1.4</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
@@ -5500,7 +5500,7 @@
     <row r="153">
       <c r="A153" s="8" t="inlineStr">
         <is>
-          <t>DQ_Phone_WSConsumer_EU_v1.4</t>
+          <t>DQ_Email_WSConsumer_US_v1.4</t>
         </is>
       </c>
       <c r="B153" s="10" t="inlineStr">
@@ -5530,7 +5530,7 @@
     <row r="154">
       <c r="A154" s="8" t="inlineStr">
         <is>
-          <t>DQ_Phone_WSConsumer_US_v1.4</t>
+          <t>DQ_Phone_WSConsumer_EU_v1.4</t>
         </is>
       </c>
       <c r="B154" s="10" t="inlineStr">
@@ -5560,7 +5560,7 @@
     <row r="155">
       <c r="A155" s="8" t="inlineStr">
         <is>
-          <t>FEP_SK</t>
+          <t>DQ_Phone_WSConsumer_US_v1.4</t>
         </is>
       </c>
       <c r="B155" s="10" t="inlineStr">
@@ -5590,7 +5590,7 @@
     <row r="156">
       <c r="A156" s="8" t="inlineStr">
         <is>
-          <t>FF_target_pooja</t>
+          <t>FEP_SK</t>
         </is>
       </c>
       <c r="B156" s="10" t="inlineStr">
@@ -5620,7 +5620,7 @@
     <row r="157">
       <c r="A157" s="8" t="inlineStr">
         <is>
-          <t>fp_nec_nandish</t>
+          <t>FF_target_pooja</t>
         </is>
       </c>
       <c r="B157" s="10" t="inlineStr">
@@ -5650,7 +5650,7 @@
     <row r="158">
       <c r="A158" s="8" t="inlineStr">
         <is>
-          <t>RestV2-AM-Login</t>
+          <t>fp_nec_nandish</t>
         </is>
       </c>
       <c r="B158" s="10" t="inlineStr">

</xml_diff>